<commit_message>
Création de rapport dois importer la saisonnalité + météo
</commit_message>
<xml_diff>
--- a/notebooks/prediction/plages_critiques.xlsx
+++ b/notebooks/prediction/plages_critiques.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F161"/>
+  <dimension ref="A1:F174"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -474,13 +474,13 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D2" t="n">
         <v>7</v>
       </c>
       <c r="E2" t="n">
-        <v>0.8621577748660575</v>
+        <v>0.852108206411805</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -490,11 +490,11 @@
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
-        <v>45292</v>
+        <v>45293</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Nuit (00–08)</t>
+          <t>Midi (12–16)</t>
         </is>
       </c>
       <c r="C3" t="n">
@@ -504,7 +504,7 @@
         <v>6</v>
       </c>
       <c r="E3" t="n">
-        <v>0.8701946590885972</v>
+        <v>0.8540205811009263</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -514,21 +514,21 @@
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
-        <v>45292</v>
+        <v>45294</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Soir (20–00)</t>
+          <t>Midi (12–16)</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D4" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E4" t="n">
-        <v>0.8848386533332595</v>
+        <v>0.8666870088288279</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -538,7 +538,7 @@
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
-        <v>45294</v>
+        <v>45295</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -546,13 +546,13 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D5" t="n">
         <v>6</v>
       </c>
       <c r="E5" t="n">
-        <v>0.8601737672632391</v>
+        <v>0.887059009436405</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
@@ -562,25 +562,25 @@
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>45295</v>
+        <v>45296</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Soir (20–00)</t>
+          <t>Après‑midi (16–20)</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D6" t="n">
         <v>7</v>
       </c>
       <c r="E6" t="n">
-        <v>0.8588235402348067</v>
+        <v>0.839584069850641</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>⚠️ Système saturé — renfort nécessaire</t>
+          <t>🔴 Forte activité</t>
         </is>
       </c>
     </row>
@@ -590,7 +590,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Après‑midi (16–20)</t>
+          <t>Soir (20–00)</t>
         </is>
       </c>
       <c r="C7" t="n">
@@ -600,7 +600,7 @@
         <v>7</v>
       </c>
       <c r="E7" t="n">
-        <v>0.8413802906548308</v>
+        <v>0.8101272961450002</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
@@ -610,11 +610,11 @@
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
-        <v>45296</v>
+        <v>45297</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Soir (20–00)</t>
+          <t>Après‑midi (16–20)</t>
         </is>
       </c>
       <c r="C8" t="n">
@@ -624,11 +624,11 @@
         <v>7</v>
       </c>
       <c r="E8" t="n">
-        <v>0.811083120701117</v>
+        <v>0.8645512049676365</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>🔴 Forte activité</t>
+          <t>⚠️ Système saturé — renfort nécessaire</t>
         </is>
       </c>
     </row>
@@ -638,17 +638,17 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Après‑midi (16–20)</t>
+          <t>Nuit (00–08)</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D9" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E9" t="n">
-        <v>0.8578269994276084</v>
+        <v>0.8654987234057803</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
@@ -662,17 +662,17 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Nuit (00–08)</t>
+          <t>Soir (20–00)</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D10" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E10" t="n">
-        <v>0.8641072475548947</v>
+        <v>0.8673520459757224</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
@@ -682,25 +682,25 @@
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
-        <v>45297</v>
+        <v>45298</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Soir (20–00)</t>
+          <t>Après‑midi (16–20)</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D11" t="n">
         <v>7</v>
       </c>
       <c r="E11" t="n">
-        <v>0.8917361269093524</v>
+        <v>0.8402986306304713</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>⚠️ Système saturé — renfort nécessaire</t>
+          <t>🔴 Forte activité</t>
         </is>
       </c>
     </row>
@@ -710,21 +710,21 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Après‑midi (16–20)</t>
+          <t>Nuit (00–08)</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D12" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E12" t="n">
-        <v>0.8246705507991291</v>
+        <v>0.8584535338661887</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>🔴 Forte activité</t>
+          <t>⚠️ Système saturé — renfort nécessaire</t>
         </is>
       </c>
     </row>
@@ -744,7 +744,7 @@
         <v>7</v>
       </c>
       <c r="E13" t="n">
-        <v>0.8340630696449446</v>
+        <v>0.8171824459389692</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
@@ -768,7 +768,7 @@
         <v>7</v>
       </c>
       <c r="E14" t="n">
-        <v>0.8199786727046554</v>
+        <v>0.8368827357436672</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
@@ -782,55 +782,55 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Soir (20–00)</t>
+          <t>Midi (12–16)</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D15" t="n">
         <v>7</v>
       </c>
       <c r="E15" t="n">
-        <v>0.8064420570714822</v>
+        <v>0.864636657213924</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>🔴 Forte activité</t>
+          <t>⚠️ Système saturé — renfort nécessaire</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
-        <v>45301</v>
+        <v>45299</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Après‑midi (16–20)</t>
+          <t>Soir (20–00)</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D16" t="n">
         <v>7</v>
       </c>
       <c r="E16" t="n">
-        <v>0.8513155730083737</v>
+        <v>0.8232739804283022</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>⚠️ Système saturé — renfort nécessaire</t>
+          <t>🔴 Forte activité</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
-        <v>45301</v>
+        <v>45300</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Soir (20–00)</t>
+          <t>Après‑midi (16–20)</t>
         </is>
       </c>
       <c r="C17" t="n">
@@ -840,7 +840,7 @@
         <v>7</v>
       </c>
       <c r="E17" t="n">
-        <v>0.8515421115990842</v>
+        <v>0.8669753026480628</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
@@ -850,21 +850,21 @@
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
-        <v>45302</v>
+        <v>45300</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Après‑midi (16–20)</t>
+          <t>Nuit (00–08)</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D18" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E18" t="n">
-        <v>0.8572462592462098</v>
+        <v>0.8557542165120443</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
@@ -874,7 +874,7 @@
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
-        <v>45302</v>
+        <v>45300</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
@@ -888,7 +888,7 @@
         <v>7</v>
       </c>
       <c r="E19" t="n">
-        <v>0.8677992772574378</v>
+        <v>0.8663223391831524</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
@@ -898,7 +898,7 @@
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
-        <v>45303</v>
+        <v>45301</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
@@ -906,23 +906,23 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D20" t="n">
         <v>7</v>
       </c>
       <c r="E20" t="n">
-        <v>0.8125462332501213</v>
+        <v>0.8665477507042163</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>🔴 Forte activité</t>
+          <t>⚠️ Système saturé — renfort nécessaire</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
-        <v>45303</v>
+        <v>45301</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
@@ -930,23 +930,23 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D21" t="n">
         <v>7</v>
       </c>
       <c r="E21" t="n">
-        <v>0.8141309375542756</v>
+        <v>0.8665700392289597</v>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>🔴 Forte activité</t>
+          <t>⚠️ Système saturé — renfort nécessaire</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
-        <v>45304</v>
+        <v>45302</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
@@ -954,13 +954,13 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D22" t="n">
         <v>7</v>
       </c>
       <c r="E22" t="n">
-        <v>0.8566224007379442</v>
+        <v>0.8715952526439321</v>
       </c>
       <c r="F22" t="inlineStr">
         <is>
@@ -970,21 +970,21 @@
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
-        <v>45304</v>
+        <v>45302</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Nuit (00–08)</t>
+          <t>Soir (20–00)</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D23" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E23" t="n">
-        <v>0.8666096456123121</v>
+        <v>0.882202957615708</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
@@ -994,35 +994,35 @@
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
-        <v>45304</v>
+        <v>45303</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Soir (20–00)</t>
+          <t>Après‑midi (16–20)</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D24" t="n">
         <v>7</v>
       </c>
       <c r="E24" t="n">
-        <v>0.8908875975945985</v>
+        <v>0.8247498172358174</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>⚠️ Système saturé — renfort nécessaire</t>
+          <t>🔴 Forte activité</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
-        <v>45305</v>
+        <v>45303</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Après‑midi (16–20)</t>
+          <t>Soir (20–00)</t>
         </is>
       </c>
       <c r="C25" t="n">
@@ -1032,7 +1032,7 @@
         <v>7</v>
       </c>
       <c r="E25" t="n">
-        <v>0.8194385049663067</v>
+        <v>0.8258543317280119</v>
       </c>
       <c r="F25" t="inlineStr">
         <is>
@@ -1042,11 +1042,11 @@
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
-        <v>45305</v>
+        <v>45304</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Soir (20–00)</t>
+          <t>Après‑midi (16–20)</t>
         </is>
       </c>
       <c r="C26" t="n">
@@ -1056,41 +1056,41 @@
         <v>7</v>
       </c>
       <c r="E26" t="n">
-        <v>0.8282907098574729</v>
+        <v>0.8672249781620969</v>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>🔴 Forte activité</t>
+          <t>⚠️ Système saturé — renfort nécessaire</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="n">
-        <v>45306</v>
+        <v>45304</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Après‑midi (16–20)</t>
+          <t>Nuit (00–08)</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D27" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E27" t="n">
-        <v>0.8143984394156056</v>
+        <v>0.8809790683515144</v>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>🔴 Forte activité</t>
+          <t>⚠️ Système saturé — renfort nécessaire</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
-        <v>45306</v>
+        <v>45304</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
@@ -1104,55 +1104,55 @@
         <v>7</v>
       </c>
       <c r="E28" t="n">
-        <v>0.8373540978755099</v>
+        <v>0.8686416448452773</v>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>🔴 Forte activité</t>
+          <t>⚠️ Système saturé — renfort nécessaire</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="n">
-        <v>45309</v>
+        <v>45305</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Soir (20–00)</t>
+          <t>Après‑midi (16–20)</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D29" t="n">
         <v>7</v>
       </c>
       <c r="E29" t="n">
-        <v>0.857708863537721</v>
+        <v>0.8293917271998023</v>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>⚠️ Système saturé — renfort nécessaire</t>
+          <t>🔴 Forte activité</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="n">
-        <v>45310</v>
+        <v>45305</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Après‑midi (16–20)</t>
+          <t>Nuit (00–08)</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D30" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E30" t="n">
-        <v>0.8682979443372587</v>
+        <v>0.8537331494418058</v>
       </c>
       <c r="F30" t="inlineStr">
         <is>
@@ -1162,7 +1162,7 @@
     </row>
     <row r="31">
       <c r="A31" s="2" t="n">
-        <v>45310</v>
+        <v>45305</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
@@ -1176,7 +1176,7 @@
         <v>7</v>
       </c>
       <c r="E31" t="n">
-        <v>0.8378607507735965</v>
+        <v>0.8382345019996942</v>
       </c>
       <c r="F31" t="inlineStr">
         <is>
@@ -1186,7 +1186,7 @@
     </row>
     <row r="32">
       <c r="A32" s="2" t="n">
-        <v>45311</v>
+        <v>45306</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
@@ -1194,37 +1194,37 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D32" t="n">
         <v>7</v>
       </c>
       <c r="E32" t="n">
-        <v>0.8791554335391883</v>
+        <v>0.8243418290329531</v>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>⚠️ Système saturé — renfort nécessaire</t>
+          <t>🔴 Forte activité</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="n">
-        <v>45311</v>
+        <v>45306</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Nuit (00–08)</t>
+          <t>Midi (12–16)</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D33" t="n">
         <v>6</v>
       </c>
       <c r="E33" t="n">
-        <v>0.853905981237238</v>
+        <v>0.8500994094694505</v>
       </c>
       <c r="F33" t="inlineStr">
         <is>
@@ -1234,7 +1234,7 @@
     </row>
     <row r="34">
       <c r="A34" s="2" t="n">
-        <v>45311</v>
+        <v>45306</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
@@ -1242,23 +1242,23 @@
         </is>
       </c>
       <c r="C34" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D34" t="n">
         <v>7</v>
       </c>
       <c r="E34" t="n">
-        <v>0.879078730188235</v>
+        <v>0.8091632060674363</v>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>⚠️ Système saturé — renfort nécessaire</t>
+          <t>🔴 Forte activité</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="n">
-        <v>45312</v>
+        <v>45307</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
@@ -1266,23 +1266,23 @@
         </is>
       </c>
       <c r="C35" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D35" t="n">
         <v>7</v>
       </c>
       <c r="E35" t="n">
-        <v>0.8441717800123868</v>
+        <v>0.8506037972190165</v>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>🔴 Forte activité</t>
+          <t>⚠️ Système saturé — renfort nécessaire</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="n">
-        <v>45312</v>
+        <v>45309</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
@@ -1290,23 +1290,23 @@
         </is>
       </c>
       <c r="C36" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D36" t="n">
         <v>7</v>
       </c>
       <c r="E36" t="n">
-        <v>0.8197976999296599</v>
+        <v>0.859142202319521</v>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>🔴 Forte activité</t>
+          <t>⚠️ Système saturé — renfort nécessaire</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="n">
-        <v>45313</v>
+        <v>45310</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
@@ -1320,7 +1320,7 @@
         <v>7</v>
       </c>
       <c r="E37" t="n">
-        <v>0.8729399678339003</v>
+        <v>0.868416868074976</v>
       </c>
       <c r="F37" t="inlineStr">
         <is>
@@ -1330,7 +1330,7 @@
     </row>
     <row r="38">
       <c r="A38" s="2" t="n">
-        <v>45313</v>
+        <v>45310</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
@@ -1338,27 +1338,27 @@
         </is>
       </c>
       <c r="C38" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D38" t="n">
         <v>7</v>
       </c>
       <c r="E38" t="n">
-        <v>0.8951306150417137</v>
+        <v>0.8367274505923494</v>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>⚠️ Système saturé — renfort nécessaire</t>
+          <t>🔴 Forte activité</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="n">
-        <v>45316</v>
+        <v>45311</v>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Soir (20–00)</t>
+          <t>Après‑midi (16–20)</t>
         </is>
       </c>
       <c r="C39" t="n">
@@ -1368,7 +1368,7 @@
         <v>7</v>
       </c>
       <c r="E39" t="n">
-        <v>0.8563380385890152</v>
+        <v>0.8754056631916702</v>
       </c>
       <c r="F39" t="inlineStr">
         <is>
@@ -1378,21 +1378,21 @@
     </row>
     <row r="40">
       <c r="A40" s="2" t="n">
-        <v>45317</v>
+        <v>45311</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Après‑midi (16–20)</t>
+          <t>Nuit (00–08)</t>
         </is>
       </c>
       <c r="C40" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D40" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E40" t="n">
-        <v>0.8687751702588015</v>
+        <v>0.8513175429719867</v>
       </c>
       <c r="F40" t="inlineStr">
         <is>
@@ -1402,7 +1402,7 @@
     </row>
     <row r="41">
       <c r="A41" s="2" t="n">
-        <v>45317</v>
+        <v>45311</v>
       </c>
       <c r="B41" t="inlineStr">
         <is>
@@ -1410,23 +1410,23 @@
         </is>
       </c>
       <c r="C41" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D41" t="n">
         <v>7</v>
       </c>
       <c r="E41" t="n">
-        <v>0.837338956403526</v>
+        <v>0.8743996475682114</v>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>🔴 Forte activité</t>
+          <t>⚠️ Système saturé — renfort nécessaire</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="n">
-        <v>45318</v>
+        <v>45312</v>
       </c>
       <c r="B42" t="inlineStr">
         <is>
@@ -1434,61 +1434,61 @@
         </is>
       </c>
       <c r="C42" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D42" t="n">
         <v>7</v>
       </c>
       <c r="E42" t="n">
-        <v>0.8807843622535168</v>
+        <v>0.8424273266592757</v>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>⚠️ Système saturé — renfort nécessaire</t>
+          <t>🔴 Forte activité</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="n">
-        <v>45318</v>
+        <v>45312</v>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Nuit (00–08)</t>
+          <t>Soir (20–00)</t>
         </is>
       </c>
       <c r="C43" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D43" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E43" t="n">
-        <v>0.8544829252994421</v>
+        <v>0.8179926803445748</v>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>⚠️ Système saturé — renfort nécessaire</t>
+          <t>🔴 Forte activité</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="n">
-        <v>45318</v>
+        <v>45313</v>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Soir (20–00)</t>
+          <t>Après‑midi (16–20)</t>
         </is>
       </c>
       <c r="C44" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D44" t="n">
         <v>7</v>
       </c>
       <c r="E44" t="n">
-        <v>0.8809372343198218</v>
+        <v>0.8732122845119902</v>
       </c>
       <c r="F44" t="inlineStr">
         <is>
@@ -1498,31 +1498,31 @@
     </row>
     <row r="45">
       <c r="A45" s="2" t="n">
-        <v>45319</v>
+        <v>45313</v>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Après‑midi (16–20)</t>
+          <t>Nuit (00–08)</t>
         </is>
       </c>
       <c r="C45" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D45" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E45" t="n">
-        <v>0.8133017208325055</v>
+        <v>0.8664334651195642</v>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>🔴 Forte activité</t>
+          <t>⚠️ Système saturé — renfort nécessaire</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="n">
-        <v>45319</v>
+        <v>45313</v>
       </c>
       <c r="B46" t="inlineStr">
         <is>
@@ -1530,51 +1530,51 @@
         </is>
       </c>
       <c r="C46" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D46" t="n">
         <v>7</v>
       </c>
       <c r="E46" t="n">
-        <v>0.8220121079537088</v>
+        <v>0.8947229289045239</v>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>🔴 Forte activité</t>
+          <t>⚠️ Système saturé — renfort nécessaire</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="n">
-        <v>45320</v>
+        <v>45315</v>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Après‑midi (16–20)</t>
+          <t>Midi (12–16)</t>
         </is>
       </c>
       <c r="C47" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D47" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E47" t="n">
-        <v>0.8102746099276633</v>
+        <v>0.8615851233703922</v>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>🔴 Forte activité</t>
+          <t>⚠️ Système saturé — renfort nécessaire</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="n">
-        <v>45320</v>
+        <v>45316</v>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Nuit (00–08)</t>
+          <t>Midi (12–16)</t>
         </is>
       </c>
       <c r="C48" t="n">
@@ -1584,7 +1584,7 @@
         <v>6</v>
       </c>
       <c r="E48" t="n">
-        <v>0.8523853330901175</v>
+        <v>0.8628019925319788</v>
       </c>
       <c r="F48" t="inlineStr">
         <is>
@@ -1594,7 +1594,7 @@
     </row>
     <row r="49">
       <c r="A49" s="2" t="n">
-        <v>45320</v>
+        <v>45316</v>
       </c>
       <c r="B49" t="inlineStr">
         <is>
@@ -1602,13 +1602,13 @@
         </is>
       </c>
       <c r="C49" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D49" t="n">
         <v>7</v>
       </c>
       <c r="E49" t="n">
-        <v>0.8667282315043661</v>
+        <v>0.8538167741563586</v>
       </c>
       <c r="F49" t="inlineStr">
         <is>
@@ -1618,7 +1618,7 @@
     </row>
     <row r="50">
       <c r="A50" s="2" t="n">
-        <v>45323</v>
+        <v>45317</v>
       </c>
       <c r="B50" t="inlineStr">
         <is>
@@ -1626,13 +1626,13 @@
         </is>
       </c>
       <c r="C50" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D50" t="n">
         <v>7</v>
       </c>
       <c r="E50" t="n">
-        <v>0.8515337500909363</v>
+        <v>0.867037501342025</v>
       </c>
       <c r="F50" t="inlineStr">
         <is>
@@ -1642,7 +1642,7 @@
     </row>
     <row r="51">
       <c r="A51" s="2" t="n">
-        <v>45323</v>
+        <v>45317</v>
       </c>
       <c r="B51" t="inlineStr">
         <is>
@@ -1650,23 +1650,23 @@
         </is>
       </c>
       <c r="C51" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D51" t="n">
         <v>7</v>
       </c>
       <c r="E51" t="n">
-        <v>0.8616224683896461</v>
+        <v>0.834685004978813</v>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>⚠️ Système saturé — renfort nécessaire</t>
+          <t>🔴 Forte activité</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="n">
-        <v>45324</v>
+        <v>45318</v>
       </c>
       <c r="B52" t="inlineStr">
         <is>
@@ -1674,61 +1674,61 @@
         </is>
       </c>
       <c r="C52" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D52" t="n">
         <v>7</v>
       </c>
       <c r="E52" t="n">
-        <v>0.8417620734562951</v>
+        <v>0.8773116631941363</v>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>🔴 Forte activité</t>
+          <t>⚠️ Système saturé — renfort nécessaire</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="n">
-        <v>45324</v>
+        <v>45318</v>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Soir (20–00)</t>
+          <t>Nuit (00–08)</t>
         </is>
       </c>
       <c r="C53" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D53" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E53" t="n">
-        <v>0.8110728459956843</v>
+        <v>0.8506751927462491</v>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>🔴 Forte activité</t>
+          <t>⚠️ Système saturé — renfort nécessaire</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="n">
-        <v>45325</v>
+        <v>45318</v>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Après‑midi (16–20)</t>
+          <t>Soir (20–00)</t>
         </is>
       </c>
       <c r="C54" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D54" t="n">
         <v>7</v>
       </c>
       <c r="E54" t="n">
-        <v>0.8553585896072279</v>
+        <v>0.8766470099940445</v>
       </c>
       <c r="F54" t="inlineStr">
         <is>
@@ -1738,31 +1738,31 @@
     </row>
     <row r="55">
       <c r="A55" s="2" t="n">
-        <v>45325</v>
+        <v>45319</v>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Nuit (00–08)</t>
+          <t>Après‑midi (16–20)</t>
         </is>
       </c>
       <c r="C55" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D55" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E55" t="n">
-        <v>0.863175139282689</v>
+        <v>0.8122016753985253</v>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>⚠️ Système saturé — renfort nécessaire</t>
+          <t>🔴 Forte activité</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="n">
-        <v>45325</v>
+        <v>45319</v>
       </c>
       <c r="B56" t="inlineStr">
         <is>
@@ -1770,23 +1770,23 @@
         </is>
       </c>
       <c r="C56" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D56" t="n">
         <v>7</v>
       </c>
       <c r="E56" t="n">
-        <v>0.8891585330770474</v>
+        <v>0.820900895034768</v>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>⚠️ Système saturé — renfort nécessaire</t>
+          <t>🔴 Forte activité</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="n">
-        <v>45326</v>
+        <v>45320</v>
       </c>
       <c r="B57" t="inlineStr">
         <is>
@@ -1800,7 +1800,7 @@
         <v>7</v>
       </c>
       <c r="E57" t="n">
-        <v>0.8213514339012158</v>
+        <v>0.8115005183529544</v>
       </c>
       <c r="F57" t="inlineStr">
         <is>
@@ -1810,35 +1810,35 @@
     </row>
     <row r="58">
       <c r="A58" s="2" t="n">
-        <v>45326</v>
+        <v>45320</v>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Soir (20–00)</t>
+          <t>Nuit (00–08)</t>
         </is>
       </c>
       <c r="C58" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D58" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E58" t="n">
-        <v>0.8312315548653211</v>
+        <v>0.8521078861120975</v>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>🔴 Forte activité</t>
+          <t>⚠️ Système saturé — renfort nécessaire</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="n">
-        <v>45327</v>
+        <v>45320</v>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Après‑midi (16–20)</t>
+          <t>Soir (20–00)</t>
         </is>
       </c>
       <c r="C59" t="n">
@@ -1848,45 +1848,45 @@
         <v>7</v>
       </c>
       <c r="E59" t="n">
-        <v>0.8202735135737609</v>
+        <v>0.8675228720275527</v>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>🔴 Forte activité</t>
+          <t>⚠️ Système saturé — renfort nécessaire</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="n">
-        <v>45327</v>
+        <v>45323</v>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Soir (20–00)</t>
+          <t>Après‑midi (16–20)</t>
         </is>
       </c>
       <c r="C60" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D60" t="n">
         <v>7</v>
       </c>
       <c r="E60" t="n">
-        <v>0.8062728779312509</v>
+        <v>0.8518881870038583</v>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>🔴 Forte activité</t>
+          <t>⚠️ Système saturé — renfort nécessaire</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="n">
-        <v>45328</v>
+        <v>45323</v>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Après‑midi (16–20)</t>
+          <t>Soir (20–00)</t>
         </is>
       </c>
       <c r="C61" t="n">
@@ -1896,7 +1896,7 @@
         <v>7</v>
       </c>
       <c r="E61" t="n">
-        <v>0.8528205601855963</v>
+        <v>0.861553481130889</v>
       </c>
       <c r="F61" t="inlineStr">
         <is>
@@ -1906,69 +1906,69 @@
     </row>
     <row r="62">
       <c r="A62" s="2" t="n">
-        <v>45328</v>
+        <v>45324</v>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Soir (20–00)</t>
+          <t>Après‑midi (16–20)</t>
         </is>
       </c>
       <c r="C62" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D62" t="n">
         <v>7</v>
       </c>
       <c r="E62" t="n">
-        <v>0.8526741952607126</v>
+        <v>0.8425849375098644</v>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>⚠️ Système saturé — renfort nécessaire</t>
+          <t>🔴 Forte activité</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="n">
-        <v>45329</v>
+        <v>45324</v>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Après‑midi (16–20)</t>
+          <t>Soir (20–00)</t>
         </is>
       </c>
       <c r="C63" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D63" t="n">
         <v>7</v>
       </c>
       <c r="E63" t="n">
-        <v>0.8568629110702362</v>
+        <v>0.810978589807926</v>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>⚠️ Système saturé — renfort nécessaire</t>
+          <t>🔴 Forte activité</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="n">
-        <v>45329</v>
+        <v>45325</v>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Soir (20–00)</t>
+          <t>Après‑midi (16–20)</t>
         </is>
       </c>
       <c r="C64" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D64" t="n">
         <v>7</v>
       </c>
       <c r="E64" t="n">
-        <v>0.857432514730126</v>
+        <v>0.8540828197033375</v>
       </c>
       <c r="F64" t="inlineStr">
         <is>
@@ -1978,21 +1978,21 @@
     </row>
     <row r="65">
       <c r="A65" s="2" t="n">
-        <v>45330</v>
+        <v>45325</v>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Après‑midi (16–20)</t>
+          <t>Nuit (00–08)</t>
         </is>
       </c>
       <c r="C65" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D65" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E65" t="n">
-        <v>0.8656731518832121</v>
+        <v>0.8623981114589807</v>
       </c>
       <c r="F65" t="inlineStr">
         <is>
@@ -2002,7 +2002,7 @@
     </row>
     <row r="66">
       <c r="A66" s="2" t="n">
-        <v>45330</v>
+        <v>45325</v>
       </c>
       <c r="B66" t="inlineStr">
         <is>
@@ -2016,7 +2016,7 @@
         <v>7</v>
       </c>
       <c r="E66" t="n">
-        <v>0.8776624660299284</v>
+        <v>0.8869921607200546</v>
       </c>
       <c r="F66" t="inlineStr">
         <is>
@@ -2026,7 +2026,7 @@
     </row>
     <row r="67">
       <c r="A67" s="2" t="n">
-        <v>45331</v>
+        <v>45326</v>
       </c>
       <c r="B67" t="inlineStr">
         <is>
@@ -2040,7 +2040,7 @@
         <v>7</v>
       </c>
       <c r="E67" t="n">
-        <v>0.8217639083642121</v>
+        <v>0.8215426848220275</v>
       </c>
       <c r="F67" t="inlineStr">
         <is>
@@ -2050,7 +2050,7 @@
     </row>
     <row r="68">
       <c r="A68" s="2" t="n">
-        <v>45331</v>
+        <v>45326</v>
       </c>
       <c r="B68" t="inlineStr">
         <is>
@@ -2064,7 +2064,7 @@
         <v>7</v>
       </c>
       <c r="E68" t="n">
-        <v>0.8239308442560282</v>
+        <v>0.8313593427512209</v>
       </c>
       <c r="F68" t="inlineStr">
         <is>
@@ -2074,7 +2074,7 @@
     </row>
     <row r="69">
       <c r="A69" s="2" t="n">
-        <v>45332</v>
+        <v>45327</v>
       </c>
       <c r="B69" t="inlineStr">
         <is>
@@ -2088,55 +2088,55 @@
         <v>7</v>
       </c>
       <c r="E69" t="n">
-        <v>0.8669810480885692</v>
+        <v>0.8221880801312336</v>
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>⚠️ Système saturé — renfort nécessaire</t>
+          <t>🔴 Forte activité</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="n">
-        <v>45332</v>
+        <v>45327</v>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Nuit (00–08)</t>
+          <t>Soir (20–00)</t>
         </is>
       </c>
       <c r="C70" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D70" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E70" t="n">
-        <v>0.8793427221702808</v>
+        <v>0.8075742219261621</v>
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>⚠️ Système saturé — renfort nécessaire</t>
+          <t>🔴 Forte activité</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="n">
-        <v>45332</v>
+        <v>45328</v>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Soir (20–00)</t>
+          <t>Après‑midi (16–20)</t>
         </is>
       </c>
       <c r="C71" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D71" t="n">
         <v>7</v>
       </c>
       <c r="E71" t="n">
-        <v>0.8691111732526948</v>
+        <v>0.8536671026788578</v>
       </c>
       <c r="F71" t="inlineStr">
         <is>
@@ -2146,45 +2146,45 @@
     </row>
     <row r="72">
       <c r="A72" s="2" t="n">
-        <v>45333</v>
+        <v>45328</v>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Après‑midi (16–20)</t>
+          <t>Soir (20–00)</t>
         </is>
       </c>
       <c r="C72" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D72" t="n">
         <v>7</v>
       </c>
       <c r="E72" t="n">
-        <v>0.8299554959692137</v>
+        <v>0.8526088348542802</v>
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>🔴 Forte activité</t>
+          <t>⚠️ Système saturé — renfort nécessaire</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="n">
-        <v>45333</v>
+        <v>45329</v>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Nuit (00–08)</t>
+          <t>Après‑midi (16–20)</t>
         </is>
       </c>
       <c r="C73" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D73" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E73" t="n">
-        <v>0.8540438016255697</v>
+        <v>0.8562650343384407</v>
       </c>
       <c r="F73" t="inlineStr">
         <is>
@@ -2194,7 +2194,7 @@
     </row>
     <row r="74">
       <c r="A74" s="2" t="n">
-        <v>45333</v>
+        <v>45329</v>
       </c>
       <c r="B74" t="inlineStr">
         <is>
@@ -2202,23 +2202,23 @@
         </is>
       </c>
       <c r="C74" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D74" t="n">
         <v>7</v>
       </c>
       <c r="E74" t="n">
-        <v>0.8386364574900267</v>
+        <v>0.8559587748363765</v>
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>🔴 Forte activité</t>
+          <t>⚠️ Système saturé — renfort nécessaire</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="n">
-        <v>45334</v>
+        <v>45330</v>
       </c>
       <c r="B75" t="inlineStr">
         <is>
@@ -2226,37 +2226,37 @@
         </is>
       </c>
       <c r="C75" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D75" t="n">
         <v>7</v>
       </c>
       <c r="E75" t="n">
-        <v>0.8254972956053279</v>
+        <v>0.8646915175698022</v>
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>🔴 Forte activité</t>
+          <t>⚠️ Système saturé — renfort nécessaire</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="n">
-        <v>45334</v>
+        <v>45330</v>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>Midi (12–16)</t>
+          <t>Soir (20–00)</t>
         </is>
       </c>
       <c r="C76" t="n">
         <v>6</v>
       </c>
       <c r="D76" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E76" t="n">
-        <v>0.8523232768280339</v>
+        <v>0.8760577500468554</v>
       </c>
       <c r="F76" t="inlineStr">
         <is>
@@ -2266,11 +2266,11 @@
     </row>
     <row r="77">
       <c r="A77" s="2" t="n">
-        <v>45334</v>
+        <v>45331</v>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>Soir (20–00)</t>
+          <t>Après‑midi (16–20)</t>
         </is>
       </c>
       <c r="C77" t="n">
@@ -2280,7 +2280,7 @@
         <v>7</v>
       </c>
       <c r="E77" t="n">
-        <v>0.8114766541325513</v>
+        <v>0.8207404905927475</v>
       </c>
       <c r="F77" t="inlineStr">
         <is>
@@ -2290,45 +2290,45 @@
     </row>
     <row r="78">
       <c r="A78" s="2" t="n">
-        <v>45335</v>
+        <v>45331</v>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>Après‑midi (16–20)</t>
+          <t>Soir (20–00)</t>
         </is>
       </c>
       <c r="C78" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D78" t="n">
         <v>7</v>
       </c>
       <c r="E78" t="n">
-        <v>0.856184441633899</v>
+        <v>0.8219792127265215</v>
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>⚠️ Système saturé — renfort nécessaire</t>
+          <t>🔴 Forte activité</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="n">
-        <v>45335</v>
+        <v>45332</v>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>Soir (20–00)</t>
+          <t>Après‑midi (16–20)</t>
         </is>
       </c>
       <c r="C79" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D79" t="n">
         <v>7</v>
       </c>
       <c r="E79" t="n">
-        <v>0.8550382960926404</v>
+        <v>0.863833816192539</v>
       </c>
       <c r="F79" t="inlineStr">
         <is>
@@ -2338,21 +2338,21 @@
     </row>
     <row r="80">
       <c r="A80" s="2" t="n">
-        <v>45336</v>
+        <v>45332</v>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>Après‑midi (16–20)</t>
+          <t>Nuit (00–08)</t>
         </is>
       </c>
       <c r="C80" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D80" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E80" t="n">
-        <v>0.8571055441191704</v>
+        <v>0.8762017163363369</v>
       </c>
       <c r="F80" t="inlineStr">
         <is>
@@ -2362,7 +2362,7 @@
     </row>
     <row r="81">
       <c r="A81" s="2" t="n">
-        <v>45336</v>
+        <v>45332</v>
       </c>
       <c r="B81" t="inlineStr">
         <is>
@@ -2376,7 +2376,7 @@
         <v>7</v>
       </c>
       <c r="E81" t="n">
-        <v>0.8586438352411445</v>
+        <v>0.8978808624575838</v>
       </c>
       <c r="F81" t="inlineStr">
         <is>
@@ -2386,7 +2386,7 @@
     </row>
     <row r="82">
       <c r="A82" s="2" t="n">
-        <v>45337</v>
+        <v>45333</v>
       </c>
       <c r="B82" t="inlineStr">
         <is>
@@ -2394,23 +2394,23 @@
         </is>
       </c>
       <c r="C82" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D82" t="n">
         <v>7</v>
       </c>
       <c r="E82" t="n">
-        <v>0.8632896885727392</v>
+        <v>0.8284656344382106</v>
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>⚠️ Système saturé — renfort nécessaire</t>
+          <t>🔴 Forte activité</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="n">
-        <v>45337</v>
+        <v>45333</v>
       </c>
       <c r="B83" t="inlineStr">
         <is>
@@ -2418,23 +2418,23 @@
         </is>
       </c>
       <c r="C83" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D83" t="n">
         <v>7</v>
       </c>
       <c r="E83" t="n">
-        <v>0.8745763229601312</v>
+        <v>0.8369910975039264</v>
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>⚠️ Système saturé — renfort nécessaire</t>
+          <t>🔴 Forte activité</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="n">
-        <v>45338</v>
+        <v>45334</v>
       </c>
       <c r="B84" t="inlineStr">
         <is>
@@ -2448,7 +2448,7 @@
         <v>7</v>
       </c>
       <c r="E84" t="n">
-        <v>0.8170422847136791</v>
+        <v>0.8257497234261915</v>
       </c>
       <c r="F84" t="inlineStr">
         <is>
@@ -2458,35 +2458,35 @@
     </row>
     <row r="85">
       <c r="A85" s="2" t="n">
-        <v>45338</v>
+        <v>45334</v>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>Soir (20–00)</t>
+          <t>Midi (12–16)</t>
         </is>
       </c>
       <c r="C85" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D85" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E85" t="n">
-        <v>0.8184805800560406</v>
+        <v>0.8516450843425714</v>
       </c>
       <c r="F85" t="inlineStr">
         <is>
-          <t>🔴 Forte activité</t>
+          <t>⚠️ Système saturé — renfort nécessaire</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="n">
-        <v>45339</v>
+        <v>45334</v>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>Après‑midi (16–20)</t>
+          <t>Soir (20–00)</t>
         </is>
       </c>
       <c r="C86" t="n">
@@ -2496,31 +2496,31 @@
         <v>7</v>
       </c>
       <c r="E86" t="n">
-        <v>0.8594509361454248</v>
+        <v>0.8110699251100615</v>
       </c>
       <c r="F86" t="inlineStr">
         <is>
-          <t>⚠️ Système saturé — renfort nécessaire</t>
+          <t>🔴 Forte activité</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="n">
-        <v>45339</v>
+        <v>45335</v>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>Nuit (00–08)</t>
+          <t>Après‑midi (16–20)</t>
         </is>
       </c>
       <c r="C87" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D87" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E87" t="n">
-        <v>0.8711256330663507</v>
+        <v>0.8552086112475156</v>
       </c>
       <c r="F87" t="inlineStr">
         <is>
@@ -2530,7 +2530,7 @@
     </row>
     <row r="88">
       <c r="A88" s="2" t="n">
-        <v>45339</v>
+        <v>45335</v>
       </c>
       <c r="B88" t="inlineStr">
         <is>
@@ -2544,7 +2544,7 @@
         <v>7</v>
       </c>
       <c r="E88" t="n">
-        <v>0.892636477345168</v>
+        <v>0.8530976073910492</v>
       </c>
       <c r="F88" t="inlineStr">
         <is>
@@ -2554,7 +2554,7 @@
     </row>
     <row r="89">
       <c r="A89" s="2" t="n">
-        <v>45340</v>
+        <v>45336</v>
       </c>
       <c r="B89" t="inlineStr">
         <is>
@@ -2562,23 +2562,23 @@
         </is>
       </c>
       <c r="C89" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D89" t="n">
         <v>7</v>
       </c>
       <c r="E89" t="n">
-        <v>0.8211241484032394</v>
+        <v>0.8547564467998467</v>
       </c>
       <c r="F89" t="inlineStr">
         <is>
-          <t>🔴 Forte activité</t>
+          <t>⚠️ Système saturé — renfort nécessaire</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="n">
-        <v>45340</v>
+        <v>45336</v>
       </c>
       <c r="B90" t="inlineStr">
         <is>
@@ -2586,23 +2586,23 @@
         </is>
       </c>
       <c r="C90" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D90" t="n">
         <v>7</v>
       </c>
       <c r="E90" t="n">
-        <v>0.8297563528085685</v>
+        <v>0.8553515540228951</v>
       </c>
       <c r="F90" t="inlineStr">
         <is>
-          <t>🔴 Forte activité</t>
+          <t>⚠️ Système saturé — renfort nécessaire</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="n">
-        <v>45341</v>
+        <v>45337</v>
       </c>
       <c r="B91" t="inlineStr">
         <is>
@@ -2610,23 +2610,23 @@
         </is>
       </c>
       <c r="C91" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D91" t="n">
         <v>7</v>
       </c>
       <c r="E91" t="n">
-        <v>0.8147502908802997</v>
+        <v>0.8606094663793391</v>
       </c>
       <c r="F91" t="inlineStr">
         <is>
-          <t>🔴 Forte activité</t>
+          <t>⚠️ Système saturé — renfort nécessaire</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="n">
-        <v>45341</v>
+        <v>45337</v>
       </c>
       <c r="B92" t="inlineStr">
         <is>
@@ -2634,13 +2634,13 @@
         </is>
       </c>
       <c r="C92" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D92" t="n">
         <v>7</v>
       </c>
       <c r="E92" t="n">
-        <v>0.8703155001520595</v>
+        <v>0.8713255699234781</v>
       </c>
       <c r="F92" t="inlineStr">
         <is>
@@ -2650,35 +2650,35 @@
     </row>
     <row r="93">
       <c r="A93" s="2" t="n">
-        <v>45344</v>
+        <v>45338</v>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>Soir (20–00)</t>
+          <t>Après‑midi (16–20)</t>
         </is>
       </c>
       <c r="C93" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D93" t="n">
         <v>7</v>
       </c>
       <c r="E93" t="n">
-        <v>0.858878174213448</v>
+        <v>0.8158134966873676</v>
       </c>
       <c r="F93" t="inlineStr">
         <is>
-          <t>⚠️ Système saturé — renfort nécessaire</t>
+          <t>🔴 Forte activité</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="n">
-        <v>45345</v>
+        <v>45338</v>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>Après‑midi (16–20)</t>
+          <t>Soir (20–00)</t>
         </is>
       </c>
       <c r="C94" t="n">
@@ -2688,7 +2688,7 @@
         <v>7</v>
       </c>
       <c r="E94" t="n">
-        <v>0.8396918949110684</v>
+        <v>0.8165394399761294</v>
       </c>
       <c r="F94" t="inlineStr">
         <is>
@@ -2698,11 +2698,11 @@
     </row>
     <row r="95">
       <c r="A95" s="2" t="n">
-        <v>45345</v>
+        <v>45339</v>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>Soir (20–00)</t>
+          <t>Après‑midi (16–20)</t>
         </is>
       </c>
       <c r="C95" t="n">
@@ -2712,31 +2712,31 @@
         <v>7</v>
       </c>
       <c r="E95" t="n">
-        <v>0.8084224072025625</v>
+        <v>0.8575958985442896</v>
       </c>
       <c r="F95" t="inlineStr">
         <is>
-          <t>🔴 Forte activité</t>
+          <t>⚠️ Système saturé — renfort nécessaire</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="n">
-        <v>45346</v>
+        <v>45339</v>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>Après‑midi (16–20)</t>
+          <t>Nuit (00–08)</t>
         </is>
       </c>
       <c r="C96" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D96" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E96" t="n">
-        <v>0.8539086743694708</v>
+        <v>0.8684752637689764</v>
       </c>
       <c r="F96" t="inlineStr">
         <is>
@@ -2746,21 +2746,21 @@
     </row>
     <row r="97">
       <c r="A97" s="2" t="n">
-        <v>45346</v>
+        <v>45339</v>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>Nuit (00–08)</t>
+          <t>Soir (20–00)</t>
         </is>
       </c>
       <c r="C97" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D97" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E97" t="n">
-        <v>0.860651767615116</v>
+        <v>0.8901080459055275</v>
       </c>
       <c r="F97" t="inlineStr">
         <is>
@@ -2770,35 +2770,35 @@
     </row>
     <row r="98">
       <c r="A98" s="2" t="n">
-        <v>45346</v>
+        <v>45340</v>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>Soir (20–00)</t>
+          <t>Après‑midi (16–20)</t>
         </is>
       </c>
       <c r="C98" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D98" t="n">
         <v>7</v>
       </c>
       <c r="E98" t="n">
-        <v>0.8878025430621523</v>
+        <v>0.8222021237768309</v>
       </c>
       <c r="F98" t="inlineStr">
         <is>
-          <t>⚠️ Système saturé — renfort nécessaire</t>
+          <t>🔴 Forte activité</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="n">
-        <v>45347</v>
+        <v>45340</v>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>Après‑midi (16–20)</t>
+          <t>Soir (20–00)</t>
         </is>
       </c>
       <c r="C99" t="n">
@@ -2808,7 +2808,7 @@
         <v>7</v>
       </c>
       <c r="E99" t="n">
-        <v>0.8202974035970405</v>
+        <v>0.8310617323733684</v>
       </c>
       <c r="F99" t="inlineStr">
         <is>
@@ -2818,11 +2818,11 @@
     </row>
     <row r="100">
       <c r="A100" s="2" t="n">
-        <v>45347</v>
+        <v>45341</v>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>Soir (20–00)</t>
+          <t>Après‑midi (16–20)</t>
         </is>
       </c>
       <c r="C100" t="n">
@@ -2832,7 +2832,7 @@
         <v>7</v>
       </c>
       <c r="E100" t="n">
-        <v>0.8299248817163114</v>
+        <v>0.818965452229994</v>
       </c>
       <c r="F100" t="inlineStr">
         <is>
@@ -2842,11 +2842,11 @@
     </row>
     <row r="101">
       <c r="A101" s="2" t="n">
-        <v>45348</v>
+        <v>45341</v>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>Après‑midi (16–20)</t>
+          <t>Soir (20–00)</t>
         </is>
       </c>
       <c r="C101" t="n">
@@ -2856,7 +2856,7 @@
         <v>7</v>
       </c>
       <c r="E101" t="n">
-        <v>0.8186758717073164</v>
+        <v>0.8416685569509972</v>
       </c>
       <c r="F101" t="inlineStr">
         <is>
@@ -2866,35 +2866,35 @@
     </row>
     <row r="102">
       <c r="A102" s="2" t="n">
-        <v>45348</v>
+        <v>45344</v>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>Soir (20–00)</t>
+          <t>Après‑midi (16–20)</t>
         </is>
       </c>
       <c r="C102" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D102" t="n">
         <v>7</v>
       </c>
       <c r="E102" t="n">
-        <v>0.8060473951942477</v>
+        <v>0.8532090138907386</v>
       </c>
       <c r="F102" t="inlineStr">
         <is>
-          <t>🔴 Forte activité</t>
+          <t>⚠️ Système saturé — renfort nécessaire</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="n">
-        <v>45349</v>
+        <v>45344</v>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>Après‑midi (16–20)</t>
+          <t>Soir (20–00)</t>
         </is>
       </c>
       <c r="C103" t="n">
@@ -2904,7 +2904,7 @@
         <v>7</v>
       </c>
       <c r="E103" t="n">
-        <v>0.8523902507743452</v>
+        <v>0.8638434939914281</v>
       </c>
       <c r="F103" t="inlineStr">
         <is>
@@ -2914,69 +2914,69 @@
     </row>
     <row r="104">
       <c r="A104" s="2" t="n">
-        <v>45349</v>
+        <v>45345</v>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>Soir (20–00)</t>
+          <t>Après‑midi (16–20)</t>
         </is>
       </c>
       <c r="C104" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D104" t="n">
         <v>7</v>
       </c>
       <c r="E104" t="n">
-        <v>0.851524136283181</v>
+        <v>0.8106761990171492</v>
       </c>
       <c r="F104" t="inlineStr">
         <is>
-          <t>⚠️ Système saturé — renfort nécessaire</t>
+          <t>🔴 Forte activité</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="n">
-        <v>45350</v>
+        <v>45345</v>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>Après‑midi (16–20)</t>
+          <t>Soir (20–00)</t>
         </is>
       </c>
       <c r="C105" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D105" t="n">
         <v>7</v>
       </c>
       <c r="E105" t="n">
-        <v>0.8568261608932959</v>
+        <v>0.8111621394301907</v>
       </c>
       <c r="F105" t="inlineStr">
         <is>
-          <t>⚠️ Système saturé — renfort nécessaire</t>
+          <t>🔴 Forte activité</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="n">
-        <v>45350</v>
+        <v>45346</v>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>Soir (20–00)</t>
+          <t>Après‑midi (16–20)</t>
         </is>
       </c>
       <c r="C106" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D106" t="n">
         <v>7</v>
       </c>
       <c r="E106" t="n">
-        <v>0.8577934178439055</v>
+        <v>0.8546660369608827</v>
       </c>
       <c r="F106" t="inlineStr">
         <is>
@@ -2986,21 +2986,21 @@
     </row>
     <row r="107">
       <c r="A107" s="2" t="n">
-        <v>45351</v>
+        <v>45346</v>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>Après‑midi (16–20)</t>
+          <t>Nuit (00–08)</t>
         </is>
       </c>
       <c r="C107" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D107" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E107" t="n">
-        <v>0.8627079592810738</v>
+        <v>0.8632238127968528</v>
       </c>
       <c r="F107" t="inlineStr">
         <is>
@@ -3010,7 +3010,7 @@
     </row>
     <row r="108">
       <c r="A108" s="2" t="n">
-        <v>45351</v>
+        <v>45346</v>
       </c>
       <c r="B108" t="inlineStr">
         <is>
@@ -3024,7 +3024,7 @@
         <v>7</v>
       </c>
       <c r="E108" t="n">
-        <v>0.8736253699871026</v>
+        <v>0.8876555182717064</v>
       </c>
       <c r="F108" t="inlineStr">
         <is>
@@ -3034,7 +3034,7 @@
     </row>
     <row r="109">
       <c r="A109" s="2" t="n">
-        <v>45352</v>
+        <v>45347</v>
       </c>
       <c r="B109" t="inlineStr">
         <is>
@@ -3048,7 +3048,7 @@
         <v>7</v>
       </c>
       <c r="E109" t="n">
-        <v>0.8172428625142593</v>
+        <v>0.8213393650357687</v>
       </c>
       <c r="F109" t="inlineStr">
         <is>
@@ -3058,7 +3058,7 @@
     </row>
     <row r="110">
       <c r="A110" s="2" t="n">
-        <v>45352</v>
+        <v>45347</v>
       </c>
       <c r="B110" t="inlineStr">
         <is>
@@ -3072,7 +3072,7 @@
         <v>7</v>
       </c>
       <c r="E110" t="n">
-        <v>0.819453030265599</v>
+        <v>0.8307482446254935</v>
       </c>
       <c r="F110" t="inlineStr">
         <is>
@@ -3082,7 +3082,7 @@
     </row>
     <row r="111">
       <c r="A111" s="2" t="n">
-        <v>45353</v>
+        <v>45348</v>
       </c>
       <c r="B111" t="inlineStr">
         <is>
@@ -3096,45 +3096,45 @@
         <v>7</v>
       </c>
       <c r="E111" t="n">
-        <v>0.8614216635237526</v>
+        <v>0.8204039694770935</v>
       </c>
       <c r="F111" t="inlineStr">
         <is>
-          <t>⚠️ Système saturé — renfort nécessaire</t>
+          <t>🔴 Forte activité</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="n">
-        <v>45353</v>
+        <v>45348</v>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>Nuit (00–08)</t>
+          <t>Soir (20–00)</t>
         </is>
       </c>
       <c r="C112" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D112" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E112" t="n">
-        <v>0.8730099562442664</v>
+        <v>0.8069967053841376</v>
       </c>
       <c r="F112" t="inlineStr">
         <is>
-          <t>⚠️ Système saturé — renfort nécessaire</t>
+          <t>🔴 Forte activité</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="n">
-        <v>45353</v>
+        <v>45349</v>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>Soir (20–00)</t>
+          <t>Après‑midi (16–20)</t>
         </is>
       </c>
       <c r="C113" t="n">
@@ -3144,7 +3144,7 @@
         <v>7</v>
       </c>
       <c r="E113" t="n">
-        <v>0.8953918351067438</v>
+        <v>0.8518774461264563</v>
       </c>
       <c r="F113" t="inlineStr">
         <is>
@@ -3154,7 +3154,7 @@
     </row>
     <row r="114">
       <c r="A114" s="2" t="n">
-        <v>45354</v>
+        <v>45350</v>
       </c>
       <c r="B114" t="inlineStr">
         <is>
@@ -3162,23 +3162,23 @@
         </is>
       </c>
       <c r="C114" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D114" t="n">
         <v>7</v>
       </c>
       <c r="E114" t="n">
-        <v>0.8241418326571908</v>
+        <v>0.8537084165245596</v>
       </c>
       <c r="F114" t="inlineStr">
         <is>
-          <t>🔴 Forte activité</t>
+          <t>⚠️ Système saturé — renfort nécessaire</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="n">
-        <v>45354</v>
+        <v>45350</v>
       </c>
       <c r="B115" t="inlineStr">
         <is>
@@ -3186,23 +3186,23 @@
         </is>
       </c>
       <c r="C115" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D115" t="n">
         <v>7</v>
       </c>
       <c r="E115" t="n">
-        <v>0.8328668104449737</v>
+        <v>0.8535023506241617</v>
       </c>
       <c r="F115" t="inlineStr">
         <is>
-          <t>🔴 Forte activité</t>
+          <t>⚠️ Système saturé — renfort nécessaire</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="n">
-        <v>45355</v>
+        <v>45351</v>
       </c>
       <c r="B116" t="inlineStr">
         <is>
@@ -3210,23 +3210,23 @@
         </is>
       </c>
       <c r="C116" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D116" t="n">
         <v>7</v>
       </c>
       <c r="E116" t="n">
-        <v>0.8191907388651355</v>
+        <v>0.8597861155114994</v>
       </c>
       <c r="F116" t="inlineStr">
         <is>
-          <t>🔴 Forte activité</t>
+          <t>⚠️ Système saturé — renfort nécessaire</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="n">
-        <v>45355</v>
+        <v>45351</v>
       </c>
       <c r="B117" t="inlineStr">
         <is>
@@ -3234,23 +3234,23 @@
         </is>
       </c>
       <c r="C117" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D117" t="n">
         <v>7</v>
       </c>
       <c r="E117" t="n">
-        <v>0.8045517727410123</v>
+        <v>0.8701379275081135</v>
       </c>
       <c r="F117" t="inlineStr">
         <is>
-          <t>🔴 Forte activité</t>
+          <t>⚠️ Système saturé — renfort nécessaire</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="n">
-        <v>45358</v>
+        <v>45352</v>
       </c>
       <c r="B118" t="inlineStr">
         <is>
@@ -3258,23 +3258,23 @@
         </is>
       </c>
       <c r="C118" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D118" t="n">
         <v>7</v>
       </c>
       <c r="E118" t="n">
-        <v>0.8551586517179857</v>
+        <v>0.8152862785526513</v>
       </c>
       <c r="F118" t="inlineStr">
         <is>
-          <t>⚠️ Système saturé — renfort nécessaire</t>
+          <t>🔴 Forte activité</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="n">
-        <v>45358</v>
+        <v>45352</v>
       </c>
       <c r="B119" t="inlineStr">
         <is>
@@ -3282,23 +3282,23 @@
         </is>
       </c>
       <c r="C119" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D119" t="n">
         <v>7</v>
       </c>
       <c r="E119" t="n">
-        <v>0.8663720699271772</v>
+        <v>0.8166861104070711</v>
       </c>
       <c r="F119" t="inlineStr">
         <is>
-          <t>⚠️ Système saturé — renfort nécessaire</t>
+          <t>🔴 Forte activité</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="n">
-        <v>45359</v>
+        <v>45353</v>
       </c>
       <c r="B120" t="inlineStr">
         <is>
@@ -3312,55 +3312,55 @@
         <v>7</v>
       </c>
       <c r="E120" t="n">
-        <v>0.8439151308409236</v>
+        <v>0.8580935947478765</v>
       </c>
       <c r="F120" t="inlineStr">
         <is>
-          <t>🔴 Forte activité</t>
+          <t>⚠️ Système saturé — renfort nécessaire</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="n">
-        <v>45359</v>
+        <v>45353</v>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>Soir (20–00)</t>
+          <t>Nuit (00–08)</t>
         </is>
       </c>
       <c r="C121" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D121" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E121" t="n">
-        <v>0.8128073721221</v>
+        <v>0.8690561814741655</v>
       </c>
       <c r="F121" t="inlineStr">
         <is>
-          <t>🔴 Forte activité</t>
+          <t>⚠️ Système saturé — renfort nécessaire</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="n">
-        <v>45360</v>
+        <v>45353</v>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>Après‑midi (16–20)</t>
+          <t>Soir (20–00)</t>
         </is>
       </c>
       <c r="C122" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D122" t="n">
         <v>7</v>
       </c>
       <c r="E122" t="n">
-        <v>0.855845744475658</v>
+        <v>0.8911597849142673</v>
       </c>
       <c r="F122" t="inlineStr">
         <is>
@@ -3370,31 +3370,31 @@
     </row>
     <row r="123">
       <c r="A123" s="2" t="n">
-        <v>45360</v>
+        <v>45354</v>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>Nuit (00–08)</t>
+          <t>Après‑midi (16–20)</t>
         </is>
       </c>
       <c r="C123" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D123" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E123" t="n">
-        <v>0.8648950909123276</v>
+        <v>0.8232963652837845</v>
       </c>
       <c r="F123" t="inlineStr">
         <is>
-          <t>⚠️ Système saturé — renfort nécessaire</t>
+          <t>🔴 Forte activité</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="n">
-        <v>45360</v>
+        <v>45354</v>
       </c>
       <c r="B124" t="inlineStr">
         <is>
@@ -3402,23 +3402,23 @@
         </is>
       </c>
       <c r="C124" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D124" t="n">
         <v>7</v>
       </c>
       <c r="E124" t="n">
-        <v>0.8895241612135762</v>
+        <v>0.8320297685708491</v>
       </c>
       <c r="F124" t="inlineStr">
         <is>
-          <t>⚠️ Système saturé — renfort nécessaire</t>
+          <t>🔴 Forte activité</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="n">
-        <v>45361</v>
+        <v>45355</v>
       </c>
       <c r="B125" t="inlineStr">
         <is>
@@ -3432,7 +3432,7 @@
         <v>7</v>
       </c>
       <c r="E125" t="n">
-        <v>0.819423074846144</v>
+        <v>0.8208849935820609</v>
       </c>
       <c r="F125" t="inlineStr">
         <is>
@@ -3442,7 +3442,7 @@
     </row>
     <row r="126">
       <c r="A126" s="2" t="n">
-        <v>45361</v>
+        <v>45355</v>
       </c>
       <c r="B126" t="inlineStr">
         <is>
@@ -3456,7 +3456,7 @@
         <v>7</v>
       </c>
       <c r="E126" t="n">
-        <v>0.8272361669361505</v>
+        <v>0.8057822293533392</v>
       </c>
       <c r="F126" t="inlineStr">
         <is>
@@ -3466,7 +3466,7 @@
     </row>
     <row r="127">
       <c r="A127" s="2" t="n">
-        <v>45362</v>
+        <v>45356</v>
       </c>
       <c r="B127" t="inlineStr">
         <is>
@@ -3474,47 +3474,47 @@
         </is>
       </c>
       <c r="C127" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D127" t="n">
         <v>7</v>
       </c>
       <c r="E127" t="n">
-        <v>0.8148344942673633</v>
+        <v>0.85010193815135</v>
       </c>
       <c r="F127" t="inlineStr">
         <is>
-          <t>🔴 Forte activité</t>
+          <t>⚠️ Système saturé — renfort nécessaire</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="n">
-        <v>45362</v>
+        <v>45357</v>
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>Soir (20–00)</t>
+          <t>Après‑midi (16–20)</t>
         </is>
       </c>
       <c r="C128" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D128" t="n">
         <v>7</v>
       </c>
       <c r="E128" t="n">
-        <v>0.8380060732622684</v>
+        <v>0.8500095328899346</v>
       </c>
       <c r="F128" t="inlineStr">
         <is>
-          <t>🔴 Forte activité</t>
+          <t>⚠️ Système saturé — renfort nécessaire</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="n">
-        <v>45365</v>
+        <v>45358</v>
       </c>
       <c r="B129" t="inlineStr">
         <is>
@@ -3528,7 +3528,7 @@
         <v>7</v>
       </c>
       <c r="E129" t="n">
-        <v>0.8519213006954002</v>
+        <v>0.8558850697796756</v>
       </c>
       <c r="F129" t="inlineStr">
         <is>
@@ -3538,7 +3538,7 @@
     </row>
     <row r="130">
       <c r="A130" s="2" t="n">
-        <v>45365</v>
+        <v>45358</v>
       </c>
       <c r="B130" t="inlineStr">
         <is>
@@ -3552,7 +3552,7 @@
         <v>7</v>
       </c>
       <c r="E130" t="n">
-        <v>0.8619712819956771</v>
+        <v>0.8666184887741553</v>
       </c>
       <c r="F130" t="inlineStr">
         <is>
@@ -3562,7 +3562,7 @@
     </row>
     <row r="131">
       <c r="A131" s="2" t="n">
-        <v>45366</v>
+        <v>45359</v>
       </c>
       <c r="B131" t="inlineStr">
         <is>
@@ -3576,7 +3576,7 @@
         <v>7</v>
       </c>
       <c r="E131" t="n">
-        <v>0.8407063091988173</v>
+        <v>0.8118265531795883</v>
       </c>
       <c r="F131" t="inlineStr">
         <is>
@@ -3586,7 +3586,7 @@
     </row>
     <row r="132">
       <c r="A132" s="2" t="n">
-        <v>45366</v>
+        <v>45359</v>
       </c>
       <c r="B132" t="inlineStr">
         <is>
@@ -3600,7 +3600,7 @@
         <v>7</v>
       </c>
       <c r="E132" t="n">
-        <v>0.8092636635465196</v>
+        <v>0.8127027122145264</v>
       </c>
       <c r="F132" t="inlineStr">
         <is>
@@ -3610,7 +3610,7 @@
     </row>
     <row r="133">
       <c r="A133" s="2" t="n">
-        <v>45367</v>
+        <v>45360</v>
       </c>
       <c r="B133" t="inlineStr">
         <is>
@@ -3618,13 +3618,13 @@
         </is>
       </c>
       <c r="C133" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D133" t="n">
         <v>7</v>
       </c>
       <c r="E133" t="n">
-        <v>0.8847908058551828</v>
+        <v>0.8548087027853875</v>
       </c>
       <c r="F133" t="inlineStr">
         <is>
@@ -3634,7 +3634,7 @@
     </row>
     <row r="134">
       <c r="A134" s="2" t="n">
-        <v>45367</v>
+        <v>45360</v>
       </c>
       <c r="B134" t="inlineStr">
         <is>
@@ -3648,7 +3648,7 @@
         <v>6</v>
       </c>
       <c r="E134" t="n">
-        <v>0.8603032357764967</v>
+        <v>0.8642206770001035</v>
       </c>
       <c r="F134" t="inlineStr">
         <is>
@@ -3658,7 +3658,7 @@
     </row>
     <row r="135">
       <c r="A135" s="2" t="n">
-        <v>45367</v>
+        <v>45360</v>
       </c>
       <c r="B135" t="inlineStr">
         <is>
@@ -3672,7 +3672,7 @@
         <v>7</v>
       </c>
       <c r="E135" t="n">
-        <v>0.8848112183387835</v>
+        <v>0.8876517372901994</v>
       </c>
       <c r="F135" t="inlineStr">
         <is>
@@ -3682,7 +3682,7 @@
     </row>
     <row r="136">
       <c r="A136" s="2" t="n">
-        <v>45368</v>
+        <v>45361</v>
       </c>
       <c r="B136" t="inlineStr">
         <is>
@@ -3696,7 +3696,7 @@
         <v>7</v>
       </c>
       <c r="E136" t="n">
-        <v>0.8155158931902822</v>
+        <v>0.8200564425745053</v>
       </c>
       <c r="F136" t="inlineStr">
         <is>
@@ -3706,7 +3706,7 @@
     </row>
     <row r="137">
       <c r="A137" s="2" t="n">
-        <v>45368</v>
+        <v>45361</v>
       </c>
       <c r="B137" t="inlineStr">
         <is>
@@ -3720,7 +3720,7 @@
         <v>7</v>
       </c>
       <c r="E137" t="n">
-        <v>0.8247272362784734</v>
+        <v>0.8278665690539032</v>
       </c>
       <c r="F137" t="inlineStr">
         <is>
@@ -3730,7 +3730,7 @@
     </row>
     <row r="138">
       <c r="A138" s="2" t="n">
-        <v>45369</v>
+        <v>45362</v>
       </c>
       <c r="B138" t="inlineStr">
         <is>
@@ -3744,7 +3744,7 @@
         <v>7</v>
       </c>
       <c r="E138" t="n">
-        <v>0.8111802840129638</v>
+        <v>0.8174354620654174</v>
       </c>
       <c r="F138" t="inlineStr">
         <is>
@@ -3754,7 +3754,7 @@
     </row>
     <row r="139">
       <c r="A139" s="2" t="n">
-        <v>45369</v>
+        <v>45362</v>
       </c>
       <c r="B139" t="inlineStr">
         <is>
@@ -3768,21 +3768,21 @@
         <v>7</v>
       </c>
       <c r="E139" t="n">
-        <v>0.867149491330762</v>
+        <v>0.8402012815379134</v>
       </c>
       <c r="F139" t="inlineStr">
         <is>
-          <t>⚠️ Système saturé — renfort nécessaire</t>
+          <t>🔴 Forte activité</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="n">
-        <v>45372</v>
+        <v>45365</v>
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>Soir (20–00)</t>
+          <t>Après‑midi (16–20)</t>
         </is>
       </c>
       <c r="C140" t="n">
@@ -3792,7 +3792,7 @@
         <v>7</v>
       </c>
       <c r="E140" t="n">
-        <v>0.8584327842250016</v>
+        <v>0.852568354269471</v>
       </c>
       <c r="F140" t="inlineStr">
         <is>
@@ -3802,35 +3802,35 @@
     </row>
     <row r="141">
       <c r="A141" s="2" t="n">
-        <v>45373</v>
+        <v>45365</v>
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>Après‑midi (16–20)</t>
+          <t>Soir (20–00)</t>
         </is>
       </c>
       <c r="C141" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D141" t="n">
         <v>7</v>
       </c>
       <c r="E141" t="n">
-        <v>0.8370201377813608</v>
+        <v>0.8620829293222139</v>
       </c>
       <c r="F141" t="inlineStr">
         <is>
-          <t>🔴 Forte activité</t>
+          <t>⚠️ Système saturé — renfort nécessaire</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="n">
-        <v>45373</v>
+        <v>45366</v>
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>Soir (20–00)</t>
+          <t>Après‑midi (16–20)</t>
         </is>
       </c>
       <c r="C142" t="n">
@@ -3840,7 +3840,7 @@
         <v>7</v>
       </c>
       <c r="E142" t="n">
-        <v>0.8383970498006582</v>
+        <v>0.8414171612451948</v>
       </c>
       <c r="F142" t="inlineStr">
         <is>
@@ -3850,45 +3850,45 @@
     </row>
     <row r="143">
       <c r="A143" s="2" t="n">
-        <v>45374</v>
+        <v>45366</v>
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>Après‑midi (16–20)</t>
+          <t>Soir (20–00)</t>
         </is>
       </c>
       <c r="C143" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D143" t="n">
         <v>7</v>
       </c>
       <c r="E143" t="n">
-        <v>0.8805159125665223</v>
+        <v>0.8090639682043167</v>
       </c>
       <c r="F143" t="inlineStr">
         <is>
-          <t>⚠️ Système saturé — renfort nécessaire</t>
+          <t>🔴 Forte activité</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="n">
-        <v>45374</v>
+        <v>45367</v>
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>Nuit (00–08)</t>
+          <t>Après‑midi (16–20)</t>
         </is>
       </c>
       <c r="C144" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D144" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E144" t="n">
-        <v>0.8559116088982784</v>
+        <v>0.8835907897563897</v>
       </c>
       <c r="F144" t="inlineStr">
         <is>
@@ -3898,21 +3898,21 @@
     </row>
     <row r="145">
       <c r="A145" s="2" t="n">
-        <v>45374</v>
+        <v>45367</v>
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>Soir (20–00)</t>
+          <t>Nuit (00–08)</t>
         </is>
       </c>
       <c r="C145" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D145" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E145" t="n">
-        <v>0.8811279306508075</v>
+        <v>0.8594837405464866</v>
       </c>
       <c r="F145" t="inlineStr">
         <is>
@@ -3922,35 +3922,35 @@
     </row>
     <row r="146">
       <c r="A146" s="2" t="n">
-        <v>45375</v>
+        <v>45367</v>
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>Après‑midi (16–20)</t>
+          <t>Soir (20–00)</t>
         </is>
       </c>
       <c r="C146" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D146" t="n">
         <v>7</v>
       </c>
       <c r="E146" t="n">
-        <v>0.8449789765593294</v>
+        <v>0.8828308076569529</v>
       </c>
       <c r="F146" t="inlineStr">
         <is>
-          <t>🔴 Forte activité</t>
+          <t>⚠️ Système saturé — renfort nécessaire</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" s="2" t="n">
-        <v>45375</v>
+        <v>45368</v>
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>Soir (20–00)</t>
+          <t>Après‑midi (16–20)</t>
         </is>
       </c>
       <c r="C147" t="n">
@@ -3960,7 +3960,7 @@
         <v>7</v>
       </c>
       <c r="E147" t="n">
-        <v>0.8212913957681148</v>
+        <v>0.8160686905765947</v>
       </c>
       <c r="F147" t="inlineStr">
         <is>
@@ -3970,11 +3970,11 @@
     </row>
     <row r="148">
       <c r="A148" s="2" t="n">
-        <v>45376</v>
+        <v>45368</v>
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>Après‑midi (16–20)</t>
+          <t>Soir (20–00)</t>
         </is>
       </c>
       <c r="C148" t="n">
@@ -3984,41 +3984,41 @@
         <v>7</v>
       </c>
       <c r="E148" t="n">
-        <v>0.8739498098519286</v>
+        <v>0.825279722310076</v>
       </c>
       <c r="F148" t="inlineStr">
         <is>
-          <t>⚠️ Système saturé — renfort nécessaire</t>
+          <t>🔴 Forte activité</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" s="2" t="n">
-        <v>45376</v>
+        <v>45369</v>
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>Nuit (00–08)</t>
+          <t>Après‑midi (16–20)</t>
         </is>
       </c>
       <c r="C149" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D149" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E149" t="n">
-        <v>0.8504822952578767</v>
+        <v>0.8136855644237084</v>
       </c>
       <c r="F149" t="inlineStr">
         <is>
-          <t>⚠️ Système saturé — renfort nécessaire</t>
+          <t>🔴 Forte activité</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="n">
-        <v>45376</v>
+        <v>45369</v>
       </c>
       <c r="B150" t="inlineStr">
         <is>
@@ -4026,13 +4026,13 @@
         </is>
       </c>
       <c r="C150" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D150" t="n">
         <v>7</v>
       </c>
       <c r="E150" t="n">
-        <v>0.8964950484458847</v>
+        <v>0.8692838130747258</v>
       </c>
       <c r="F150" t="inlineStr">
         <is>
@@ -4042,7 +4042,7 @@
     </row>
     <row r="151">
       <c r="A151" s="2" t="n">
-        <v>45379</v>
+        <v>45372</v>
       </c>
       <c r="B151" t="inlineStr">
         <is>
@@ -4056,7 +4056,7 @@
         <v>7</v>
       </c>
       <c r="E151" t="n">
-        <v>0.8543207958491162</v>
+        <v>0.8584647274980642</v>
       </c>
       <c r="F151" t="inlineStr">
         <is>
@@ -4066,7 +4066,7 @@
     </row>
     <row r="152">
       <c r="A152" s="2" t="n">
-        <v>45380</v>
+        <v>45373</v>
       </c>
       <c r="B152" t="inlineStr">
         <is>
@@ -4080,7 +4080,7 @@
         <v>7</v>
       </c>
       <c r="E152" t="n">
-        <v>0.8658817251351318</v>
+        <v>0.8704720327864479</v>
       </c>
       <c r="F152" t="inlineStr">
         <is>
@@ -4090,7 +4090,7 @@
     </row>
     <row r="153">
       <c r="A153" s="2" t="n">
-        <v>45380</v>
+        <v>45373</v>
       </c>
       <c r="B153" t="inlineStr">
         <is>
@@ -4104,7 +4104,7 @@
         <v>7</v>
       </c>
       <c r="E153" t="n">
-        <v>0.8354836624938173</v>
+        <v>0.8380611169905891</v>
       </c>
       <c r="F153" t="inlineStr">
         <is>
@@ -4114,7 +4114,7 @@
     </row>
     <row r="154">
       <c r="A154" s="2" t="n">
-        <v>45381</v>
+        <v>45374</v>
       </c>
       <c r="B154" t="inlineStr">
         <is>
@@ -4128,7 +4128,7 @@
         <v>7</v>
       </c>
       <c r="E154" t="n">
-        <v>0.8773338915121677</v>
+        <v>0.8792163386489407</v>
       </c>
       <c r="F154" t="inlineStr">
         <is>
@@ -4138,7 +4138,7 @@
     </row>
     <row r="155">
       <c r="A155" s="2" t="n">
-        <v>45381</v>
+        <v>45374</v>
       </c>
       <c r="B155" t="inlineStr">
         <is>
@@ -4152,7 +4152,7 @@
         <v>6</v>
       </c>
       <c r="E155" t="n">
-        <v>0.8514431317647299</v>
+        <v>0.8549770225178112</v>
       </c>
       <c r="F155" t="inlineStr">
         <is>
@@ -4162,7 +4162,7 @@
     </row>
     <row r="156">
       <c r="A156" s="2" t="n">
-        <v>45381</v>
+        <v>45374</v>
       </c>
       <c r="B156" t="inlineStr">
         <is>
@@ -4176,7 +4176,7 @@
         <v>7</v>
       </c>
       <c r="E156" t="n">
-        <v>0.8765641896411627</v>
+        <v>0.8790413442284171</v>
       </c>
       <c r="F156" t="inlineStr">
         <is>
@@ -4186,7 +4186,7 @@
     </row>
     <row r="157">
       <c r="A157" s="2" t="n">
-        <v>45382</v>
+        <v>45375</v>
       </c>
       <c r="B157" t="inlineStr">
         <is>
@@ -4200,7 +4200,7 @@
         <v>7</v>
       </c>
       <c r="E157" t="n">
-        <v>0.8418595876872627</v>
+        <v>0.8126110535163384</v>
       </c>
       <c r="F157" t="inlineStr">
         <is>
@@ -4210,7 +4210,7 @@
     </row>
     <row r="158">
       <c r="A158" s="2" t="n">
-        <v>45382</v>
+        <v>45375</v>
       </c>
       <c r="B158" t="inlineStr">
         <is>
@@ -4224,7 +4224,7 @@
         <v>7</v>
       </c>
       <c r="E158" t="n">
-        <v>0.8170392537357832</v>
+        <v>0.8217286065887408</v>
       </c>
       <c r="F158" t="inlineStr">
         <is>
@@ -4234,7 +4234,7 @@
     </row>
     <row r="159">
       <c r="A159" s="2" t="n">
-        <v>45383</v>
+        <v>45376</v>
       </c>
       <c r="B159" t="inlineStr">
         <is>
@@ -4248,17 +4248,17 @@
         <v>7</v>
       </c>
       <c r="E159" t="n">
-        <v>0.8697765351717951</v>
+        <v>0.8435908953348796</v>
       </c>
       <c r="F159" t="inlineStr">
         <is>
-          <t>⚠️ Système saturé — renfort nécessaire</t>
+          <t>🔴 Forte activité</t>
         </is>
       </c>
     </row>
     <row r="160">
       <c r="A160" s="2" t="n">
-        <v>45383</v>
+        <v>45376</v>
       </c>
       <c r="B160" t="inlineStr">
         <is>
@@ -4266,13 +4266,13 @@
         </is>
       </c>
       <c r="C160" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D160" t="n">
         <v>6</v>
       </c>
       <c r="E160" t="n">
-        <v>0.8833365946105032</v>
+        <v>0.8520033046452686</v>
       </c>
       <c r="F160" t="inlineStr">
         <is>
@@ -4282,23 +4282,335 @@
     </row>
     <row r="161">
       <c r="A161" s="2" t="n">
+        <v>45376</v>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>Soir (20–00)</t>
+        </is>
+      </c>
+      <c r="C161" t="n">
+        <v>7</v>
+      </c>
+      <c r="D161" t="n">
+        <v>7</v>
+      </c>
+      <c r="E161" t="n">
+        <v>0.8656985811340862</v>
+      </c>
+      <c r="F161" t="inlineStr">
+        <is>
+          <t>⚠️ Système saturé — renfort nécessaire</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" s="2" t="n">
+        <v>45378</v>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>Midi (12–16)</t>
+        </is>
+      </c>
+      <c r="C162" t="n">
+        <v>6</v>
+      </c>
+      <c r="D162" t="n">
+        <v>6</v>
+      </c>
+      <c r="E162" t="n">
+        <v>0.8632287930960607</v>
+      </c>
+      <c r="F162" t="inlineStr">
+        <is>
+          <t>⚠️ Système saturé — renfort nécessaire</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" s="2" t="n">
+        <v>45379</v>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>Midi (12–16)</t>
+        </is>
+      </c>
+      <c r="C163" t="n">
+        <v>6</v>
+      </c>
+      <c r="D163" t="n">
+        <v>6</v>
+      </c>
+      <c r="E163" t="n">
+        <v>0.8630796658872354</v>
+      </c>
+      <c r="F163" t="inlineStr">
+        <is>
+          <t>⚠️ Système saturé — renfort nécessaire</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" s="2" t="n">
+        <v>45379</v>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>Soir (20–00)</t>
+        </is>
+      </c>
+      <c r="C164" t="n">
+        <v>6</v>
+      </c>
+      <c r="D164" t="n">
+        <v>7</v>
+      </c>
+      <c r="E164" t="n">
+        <v>0.8542286362310854</v>
+      </c>
+      <c r="F164" t="inlineStr">
+        <is>
+          <t>⚠️ Système saturé — renfort nécessaire</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" s="2" t="n">
+        <v>45380</v>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>Après‑midi (16–20)</t>
+        </is>
+      </c>
+      <c r="C165" t="n">
+        <v>7</v>
+      </c>
+      <c r="D165" t="n">
+        <v>7</v>
+      </c>
+      <c r="E165" t="n">
+        <v>0.8663572721495085</v>
+      </c>
+      <c r="F165" t="inlineStr">
+        <is>
+          <t>⚠️ Système saturé — renfort nécessaire</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" s="2" t="n">
+        <v>45380</v>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>Soir (20–00)</t>
+        </is>
+      </c>
+      <c r="C166" t="n">
+        <v>7</v>
+      </c>
+      <c r="D166" t="n">
+        <v>7</v>
+      </c>
+      <c r="E166" t="n">
+        <v>0.8350755504371457</v>
+      </c>
+      <c r="F166" t="inlineStr">
+        <is>
+          <t>🔴 Forte activité</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" s="2" t="n">
+        <v>45381</v>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>Après‑midi (16–20)</t>
+        </is>
+      </c>
+      <c r="C167" t="n">
+        <v>6</v>
+      </c>
+      <c r="D167" t="n">
+        <v>7</v>
+      </c>
+      <c r="E167" t="n">
+        <v>0.8759506061823682</v>
+      </c>
+      <c r="F167" t="inlineStr">
+        <is>
+          <t>⚠️ Système saturé — renfort nécessaire</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" s="2" t="n">
+        <v>45381</v>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>Nuit (00–08)</t>
+        </is>
+      </c>
+      <c r="C168" t="n">
+        <v>5</v>
+      </c>
+      <c r="D168" t="n">
+        <v>6</v>
+      </c>
+      <c r="E168" t="n">
+        <v>0.8503928545749548</v>
+      </c>
+      <c r="F168" t="inlineStr">
+        <is>
+          <t>⚠️ Système saturé — renfort nécessaire</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" s="2" t="n">
+        <v>45381</v>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>Soir (20–00)</t>
+        </is>
+      </c>
+      <c r="C169" t="n">
+        <v>6</v>
+      </c>
+      <c r="D169" t="n">
+        <v>7</v>
+      </c>
+      <c r="E169" t="n">
+        <v>0.8743586829214386</v>
+      </c>
+      <c r="F169" t="inlineStr">
+        <is>
+          <t>⚠️ Système saturé — renfort nécessaire</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" s="2" t="n">
+        <v>45382</v>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>Après‑midi (16–20)</t>
+        </is>
+      </c>
+      <c r="C170" t="n">
+        <v>7</v>
+      </c>
+      <c r="D170" t="n">
+        <v>7</v>
+      </c>
+      <c r="E170" t="n">
+        <v>0.8422861195573904</v>
+      </c>
+      <c r="F170" t="inlineStr">
+        <is>
+          <t>🔴 Forte activité</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" s="2" t="n">
+        <v>45382</v>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>Soir (20–00)</t>
+        </is>
+      </c>
+      <c r="C171" t="n">
+        <v>7</v>
+      </c>
+      <c r="D171" t="n">
+        <v>7</v>
+      </c>
+      <c r="E171" t="n">
+        <v>0.8173860013915004</v>
+      </c>
+      <c r="F171" t="inlineStr">
+        <is>
+          <t>🔴 Forte activité</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" s="2" t="n">
         <v>45383</v>
       </c>
-      <c r="B161" t="inlineStr">
-        <is>
-          <t>Soir (20–00)</t>
-        </is>
-      </c>
-      <c r="C161" t="n">
-        <v>6</v>
-      </c>
-      <c r="D161" t="n">
-        <v>7</v>
-      </c>
-      <c r="E161" t="n">
-        <v>0.8918962478637696</v>
-      </c>
-      <c r="F161" t="inlineStr">
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>Après‑midi (16–20)</t>
+        </is>
+      </c>
+      <c r="C172" t="n">
+        <v>7</v>
+      </c>
+      <c r="D172" t="n">
+        <v>7</v>
+      </c>
+      <c r="E172" t="n">
+        <v>0.872279414194831</v>
+      </c>
+      <c r="F172" t="inlineStr">
+        <is>
+          <t>⚠️ Système saturé — renfort nécessaire</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" s="2" t="n">
+        <v>45383</v>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>Nuit (00–08)</t>
+        </is>
+      </c>
+      <c r="C173" t="n">
+        <v>5</v>
+      </c>
+      <c r="D173" t="n">
+        <v>6</v>
+      </c>
+      <c r="E173" t="n">
+        <v>0.884754144784176</v>
+      </c>
+      <c r="F173" t="inlineStr">
+        <is>
+          <t>⚠️ Système saturé — renfort nécessaire</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" s="2" t="n">
+        <v>45383</v>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>Soir (20–00)</t>
+        </is>
+      </c>
+      <c r="C174" t="n">
+        <v>6</v>
+      </c>
+      <c r="D174" t="n">
+        <v>7</v>
+      </c>
+      <c r="E174" t="n">
+        <v>0.8939096277410334</v>
+      </c>
+      <c r="F174" t="inlineStr">
         <is>
           <t>⚠️ Système saturé — renfort nécessaire</t>
         </is>

</xml_diff>